<commit_message>
Pembaruan sistem RESIK BUMDes - 19/10/2026 12:37:57,24
</commit_message>
<xml_diff>
--- a/Template_Import_Pelanggan_RESIK_BUMDes.xlsx
+++ b/Template_Import_Pelanggan_RESIK_BUMDes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CODEX\antigrafity\revik bumdes v4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E4E398E8-BD1F-4169-819E-A03C0095A7D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1FDC18C-6A0B-4B68-81A9-D585BC82BC53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template RESIK" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2059" uniqueCount="617">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2116" uniqueCount="674">
   <si>
     <t>Nama Pelanggan</t>
   </si>
@@ -1871,6 +1871,177 @@
   </si>
   <si>
     <t>7°19'35.70"S 110°27'44.22"E</t>
+  </si>
+  <si>
+    <t>7°19'54.52"S 110°27'44.49"E</t>
+  </si>
+  <si>
+    <t>7°19'54.10"S 110°27'44.38"E</t>
+  </si>
+  <si>
+    <t>7°19'54.00"S 110°27'44.30"E</t>
+  </si>
+  <si>
+    <t>7°19'53.76"S 110°27'44.29"E</t>
+  </si>
+  <si>
+    <t>7°19'53.11"S 110°27'45.05"E</t>
+  </si>
+  <si>
+    <t>7°19'53.86"S 110°27'44.80"E</t>
+  </si>
+  <si>
+    <t>7°19'52.73"S 110°27'44.13"E</t>
+  </si>
+  <si>
+    <t>7°19'51.59"S 110°27'44.00"E</t>
+  </si>
+  <si>
+    <t>7°19'51.04"S 110°27'44.18"E</t>
+  </si>
+  <si>
+    <t>7°19'50.44"S 110°27'44.16"E</t>
+  </si>
+  <si>
+    <t>7°19'50.01"S 110°27'43.75"E</t>
+  </si>
+  <si>
+    <t>7°19'49.65"S 110°27'43.40"E</t>
+  </si>
+  <si>
+    <t>7°19'49.29"S 110°27'43.41"E</t>
+  </si>
+  <si>
+    <t>7°19'51.63"S 110°27'45.90"E</t>
+  </si>
+  <si>
+    <t>7°19'51.68"S 110°27'46.41"E</t>
+  </si>
+  <si>
+    <t>7°19'51.70"S 110°27'46.53"E</t>
+  </si>
+  <si>
+    <t>7°19'50.57"S 110°27'46.56"E</t>
+  </si>
+  <si>
+    <t>7°19'50.66"S 110°27'46.77"E</t>
+  </si>
+  <si>
+    <t>7°19'50.95"S 110°27'47.68"E</t>
+  </si>
+  <si>
+    <t>7°19'50.75"S 110°27'47.89"E</t>
+  </si>
+  <si>
+    <t>7°19'50.41"S 110°27'47.85"E</t>
+  </si>
+  <si>
+    <t>7°19'51.89"S 110°27'48.10"E</t>
+  </si>
+  <si>
+    <t>7°19'52.51"S 110°27'48.09"E</t>
+  </si>
+  <si>
+    <t>7°19'55.54"S 110°27'46.40"E</t>
+  </si>
+  <si>
+    <t>7°19'55.07"S 110°27'46.62"E</t>
+  </si>
+  <si>
+    <t>7°19'55.16"S 110°27'46.15"E</t>
+  </si>
+  <si>
+    <t>7°19'55.40"S 110°27'45.65"E</t>
+  </si>
+  <si>
+    <t>7°19'55.39"S 110°27'45.39"E</t>
+  </si>
+  <si>
+    <t>7°19'55.15"S 110°27'45.91"E</t>
+  </si>
+  <si>
+    <t>7°19'54.52"S 110°27'46.30"E</t>
+  </si>
+  <si>
+    <t>7°19'54.30"S 110°27'46.17"E</t>
+  </si>
+  <si>
+    <t>7°19'54.32"S 110°27'46.30"E</t>
+  </si>
+  <si>
+    <t>7°19'53.88"S 110°27'45.92"E</t>
+  </si>
+  <si>
+    <t>7°19'53.14"S 110°27'45.44"E</t>
+  </si>
+  <si>
+    <t>7°19'51.51"S 110°27'45.18"E</t>
+  </si>
+  <si>
+    <t>7°19'52.79"S 110°27'45.43"E</t>
+  </si>
+  <si>
+    <t>7°19'51.57"S 110°27'42.53"E</t>
+  </si>
+  <si>
+    <t>7°19'51.02"S 110°27'41.19"E</t>
+  </si>
+  <si>
+    <t>7°19'51.07"S 110°27'42.06"E</t>
+  </si>
+  <si>
+    <t>7°19'51.09"S 110°27'42.54"E</t>
+  </si>
+  <si>
+    <t>7°19'51.36"S 110°27'43.14"E</t>
+  </si>
+  <si>
+    <t>7°19'53.04"S 110°27'45.22"E</t>
+  </si>
+  <si>
+    <t>7°19'48.89"S 110°27'43.57"E</t>
+  </si>
+  <si>
+    <t>7°19'30.51"S 110°27'57.18"E</t>
+  </si>
+  <si>
+    <t>7°19'25.10"S 110°27'54.76"E</t>
+  </si>
+  <si>
+    <t>7°19'28.41"S 110°27'47.35"E</t>
+  </si>
+  <si>
+    <t>7°19'34.28"S 110°27'55.30"E</t>
+  </si>
+  <si>
+    <t>7°19'39.57"S 110°28'07.84"E</t>
+  </si>
+  <si>
+    <t>7°19'40.58"S 110°28'07.63"E</t>
+  </si>
+  <si>
+    <t>7°19'35.83"S 110°28'08.30"E</t>
+  </si>
+  <si>
+    <t>7°19'36.92"S 110°28'08.41"E</t>
+  </si>
+  <si>
+    <t>7°19'35.97"S 110°28'05.39"E</t>
+  </si>
+  <si>
+    <t>7°19'37.24"S 110°28'09.68"E</t>
+  </si>
+  <si>
+    <t>7°19'30.66"S 110°27'56.57"E</t>
+  </si>
+  <si>
+    <t>7°19'30.62"S 110°27'56.32"E</t>
+  </si>
+  <si>
+    <t>7°19'33.84"S 110°27'57.32"E</t>
+  </si>
+  <si>
+    <t>7°19'33.77"S 110°28'00.61"E</t>
   </si>
 </sst>
 </file>
@@ -2250,6 +2421,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K275"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="28.69921875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -5738,7 +5912,9 @@
       <c r="H123" s="1">
         <v>20000</v>
       </c>
-      <c r="I123" s="1"/>
+      <c r="I123" s="1" t="s">
+        <v>617</v>
+      </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A124" s="1" t="s">
@@ -5765,7 +5941,9 @@
       <c r="H124" s="1">
         <v>20000</v>
       </c>
-      <c r="I124" s="1"/>
+      <c r="I124" s="1" t="s">
+        <v>655</v>
+      </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A125" s="1" t="s">
@@ -5792,7 +5970,9 @@
       <c r="H125" s="1">
         <v>20000</v>
       </c>
-      <c r="I125" s="1"/>
+      <c r="I125" s="1" t="s">
+        <v>627</v>
+      </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A126" s="1" t="s">
@@ -5819,7 +5999,9 @@
       <c r="H126" s="1">
         <v>20000</v>
       </c>
-      <c r="I126" s="1"/>
+      <c r="I126" s="1" t="s">
+        <v>653</v>
+      </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A127" s="1" t="s">
@@ -5846,7 +6028,9 @@
       <c r="H127" s="1">
         <v>20000</v>
       </c>
-      <c r="I127" s="1"/>
+      <c r="I127" s="1" t="s">
+        <v>654</v>
+      </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A128" s="1" t="s">
@@ -5873,7 +6057,9 @@
       <c r="H128" s="1">
         <v>20000</v>
       </c>
-      <c r="I128" s="1"/>
+      <c r="I128" s="1" t="s">
+        <v>657</v>
+      </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
@@ -5900,7 +6086,9 @@
       <c r="H129" s="1">
         <v>20000</v>
       </c>
-      <c r="I129" s="1"/>
+      <c r="I129" s="1" t="s">
+        <v>625</v>
+      </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
@@ -5927,7 +6115,9 @@
       <c r="H130" s="1">
         <v>20000</v>
       </c>
-      <c r="I130" s="1"/>
+      <c r="I130" s="1" t="s">
+        <v>629</v>
+      </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A131" s="1" t="s">
@@ -5954,7 +6144,9 @@
       <c r="H131" s="1">
         <v>20000</v>
       </c>
-      <c r="I131" s="1"/>
+      <c r="I131" s="1" t="s">
+        <v>658</v>
+      </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A132" s="1" t="s">
@@ -5981,7 +6173,9 @@
       <c r="H132" s="1">
         <v>20000</v>
       </c>
-      <c r="I132" s="1"/>
+      <c r="I132" s="1" t="s">
+        <v>623</v>
+      </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A133" s="1" t="s">
@@ -6008,7 +6202,9 @@
       <c r="H133" s="1">
         <v>20000</v>
       </c>
-      <c r="I133" s="1"/>
+      <c r="I133" s="1" t="s">
+        <v>619</v>
+      </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A134" s="1" t="s">
@@ -6035,7 +6231,9 @@
       <c r="H134" s="1">
         <v>20000</v>
       </c>
-      <c r="I134" s="1"/>
+      <c r="I134" s="1" t="s">
+        <v>640</v>
+      </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A135" s="1" t="s">
@@ -6062,7 +6260,9 @@
       <c r="H135" s="1">
         <v>20000</v>
       </c>
-      <c r="I135" s="1"/>
+      <c r="I135" s="1" t="s">
+        <v>644</v>
+      </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A136" s="1" t="s">
@@ -6089,7 +6289,9 @@
       <c r="H136" s="1">
         <v>20000</v>
       </c>
-      <c r="I136" s="1"/>
+      <c r="I136" s="1" t="s">
+        <v>656</v>
+      </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A137" s="1" t="s">
@@ -6116,7 +6318,9 @@
       <c r="H137" s="1">
         <v>20000</v>
       </c>
-      <c r="I137" s="1"/>
+      <c r="I137" s="1" t="s">
+        <v>643</v>
+      </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A138" s="1" t="s">
@@ -6143,7 +6347,9 @@
       <c r="H138" s="1">
         <v>20000</v>
       </c>
-      <c r="I138" s="1"/>
+      <c r="I138" s="1" t="s">
+        <v>626</v>
+      </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A139" s="1" t="s">
@@ -6170,7 +6376,9 @@
       <c r="H139" s="1">
         <v>20000</v>
       </c>
-      <c r="I139" s="1"/>
+      <c r="I139" s="1" t="s">
+        <v>620</v>
+      </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A140" s="1" t="s">
@@ -6197,7 +6405,9 @@
       <c r="H140" s="1">
         <v>20000</v>
       </c>
-      <c r="I140" s="1"/>
+      <c r="I140" s="1" t="s">
+        <v>659</v>
+      </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A141" s="1" t="s">
@@ -6278,7 +6488,9 @@
       <c r="H143" s="1">
         <v>20000</v>
       </c>
-      <c r="I143" s="1"/>
+      <c r="I143" s="1" t="s">
+        <v>628</v>
+      </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A144" s="1" t="s">
@@ -6332,7 +6544,9 @@
       <c r="H145" s="1">
         <v>20000</v>
       </c>
-      <c r="I145" s="1"/>
+      <c r="I145" s="1" t="s">
+        <v>618</v>
+      </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A146" s="1" t="s">
@@ -6417,7 +6631,9 @@
       <c r="H148" s="1">
         <v>20000</v>
       </c>
-      <c r="I148" s="1"/>
+      <c r="I148" s="1" t="s">
+        <v>642</v>
+      </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A149" s="1" t="s">
@@ -6444,7 +6660,9 @@
       <c r="H149" s="1">
         <v>20000</v>
       </c>
-      <c r="I149" s="1"/>
+      <c r="I149" s="1" t="s">
+        <v>622</v>
+      </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A150" s="1" t="s">
@@ -6498,7 +6716,9 @@
       <c r="H151" s="1">
         <v>20000</v>
       </c>
-      <c r="I151" s="1"/>
+      <c r="I151" s="1" t="s">
+        <v>641</v>
+      </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A152" s="1" t="s">
@@ -6554,7 +6774,9 @@
       <c r="H153" s="1">
         <v>20000</v>
       </c>
-      <c r="I153" s="1"/>
+      <c r="I153" s="1" t="s">
+        <v>647</v>
+      </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A154" s="1" t="s">
@@ -6581,7 +6803,9 @@
       <c r="H154" s="1">
         <v>20000</v>
       </c>
-      <c r="I154" s="1"/>
+      <c r="I154" s="1" t="s">
+        <v>646</v>
+      </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A155" s="1" t="s">
@@ -6722,7 +6946,9 @@
       <c r="H159" s="1">
         <v>20000</v>
       </c>
-      <c r="I159" s="1"/>
+      <c r="I159" s="1" t="s">
+        <v>648</v>
+      </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A160" s="1" t="s">
@@ -6805,7 +7031,9 @@
       <c r="H162" s="1">
         <v>20000</v>
       </c>
-      <c r="I162" s="1"/>
+      <c r="I162" s="1" t="s">
+        <v>645</v>
+      </c>
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A163" s="1" t="s">
@@ -6832,7 +7060,9 @@
       <c r="H163" s="1">
         <v>20000</v>
       </c>
-      <c r="I163" s="1"/>
+      <c r="I163" s="1" t="s">
+        <v>621</v>
+      </c>
     </row>
     <row r="164" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A164" s="1" t="s">
@@ -6859,7 +7089,9 @@
       <c r="H164" s="1">
         <v>20000</v>
       </c>
-      <c r="I164" s="1"/>
+      <c r="I164" s="1" t="s">
+        <v>649</v>
+      </c>
     </row>
     <row r="165" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A165" s="1" t="s">
@@ -6886,7 +7118,9 @@
       <c r="H165" s="1">
         <v>20000</v>
       </c>
-      <c r="I165" s="1"/>
+      <c r="I165" s="1" t="s">
+        <v>650</v>
+      </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A166" s="1" t="s">
@@ -6969,7 +7203,9 @@
       <c r="H168" s="1">
         <v>20000</v>
       </c>
-      <c r="I168" s="1"/>
+      <c r="I168" s="1" t="s">
+        <v>632</v>
+      </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A169" s="1" t="s">
@@ -6996,7 +7232,9 @@
       <c r="H169" s="1">
         <v>20000</v>
       </c>
-      <c r="I169" s="1"/>
+      <c r="I169" s="1" t="s">
+        <v>635</v>
+      </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A170" s="1" t="s">
@@ -7023,7 +7261,9 @@
       <c r="H170" s="1">
         <v>20000</v>
       </c>
-      <c r="I170" s="1"/>
+      <c r="I170" s="1" t="s">
+        <v>634</v>
+      </c>
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A171" s="1" t="s">
@@ -7050,7 +7290,9 @@
       <c r="H171" s="1">
         <v>20000</v>
       </c>
-      <c r="I171" s="1"/>
+      <c r="I171" s="1" t="s">
+        <v>637</v>
+      </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A172" s="1" t="s">
@@ -7077,7 +7319,9 @@
       <c r="H172" s="1">
         <v>20000</v>
       </c>
-      <c r="I172" s="1"/>
+      <c r="I172" s="1" t="s">
+        <v>636</v>
+      </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A173" s="1" t="s">
@@ -7104,7 +7348,9 @@
       <c r="H173" s="1">
         <v>20000</v>
       </c>
-      <c r="I173" s="1"/>
+      <c r="I173" s="1" t="s">
+        <v>631</v>
+      </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A174" s="1" t="s">
@@ -7131,7 +7377,9 @@
       <c r="H174" s="1">
         <v>20000</v>
       </c>
-      <c r="I174" s="1"/>
+      <c r="I174" s="1" t="s">
+        <v>639</v>
+      </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A175" s="1" t="s">
@@ -7158,7 +7406,9 @@
       <c r="H175" s="1">
         <v>20000</v>
       </c>
-      <c r="I175" s="1"/>
+      <c r="I175" s="1" t="s">
+        <v>633</v>
+      </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A176" s="1" t="s">
@@ -7185,7 +7435,9 @@
       <c r="H176" s="1">
         <v>20000</v>
       </c>
-      <c r="I176" s="1"/>
+      <c r="I176" s="1" t="s">
+        <v>651</v>
+      </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A177" s="1" t="s">
@@ -7212,7 +7464,9 @@
       <c r="H177" s="1">
         <v>20000</v>
       </c>
-      <c r="I177" s="1"/>
+      <c r="I177" s="1" t="s">
+        <v>630</v>
+      </c>
     </row>
     <row r="178" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A178" s="1" t="s">
@@ -7239,7 +7493,9 @@
       <c r="H178" s="1">
         <v>20000</v>
       </c>
-      <c r="I178" s="1"/>
+      <c r="I178" s="1" t="s">
+        <v>652</v>
+      </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A179" s="1" t="s">
@@ -7293,7 +7549,9 @@
       <c r="H180" s="1">
         <v>20000</v>
       </c>
-      <c r="I180" s="1"/>
+      <c r="I180" s="1" t="s">
+        <v>638</v>
+      </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A181" s="1" t="s">
@@ -7347,7 +7605,9 @@
       <c r="H182" s="1">
         <v>20000</v>
       </c>
-      <c r="I182" s="1"/>
+      <c r="I182" s="1" t="s">
+        <v>624</v>
+      </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A183" s="1" t="s">
@@ -8570,7 +8830,9 @@
       <c r="H225" s="1">
         <v>20000</v>
       </c>
-      <c r="I225" s="1"/>
+      <c r="I225" s="1" t="s">
+        <v>672</v>
+      </c>
     </row>
     <row r="226" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A226" s="1" t="s">
@@ -8713,7 +8975,9 @@
       <c r="H230" s="1">
         <v>20000</v>
       </c>
-      <c r="I230" s="1"/>
+      <c r="I230" s="1" t="s">
+        <v>660</v>
+      </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A231" s="1" t="s">
@@ -8740,7 +9004,9 @@
       <c r="H231" s="1">
         <v>20000</v>
       </c>
-      <c r="I231" s="1"/>
+      <c r="I231" s="1" t="s">
+        <v>661</v>
+      </c>
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A232" s="1" t="s">
@@ -8767,7 +9033,9 @@
       <c r="H232" s="1">
         <v>20000</v>
       </c>
-      <c r="I232" s="1"/>
+      <c r="I232" s="1" t="s">
+        <v>662</v>
+      </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A233" s="1" t="s">
@@ -8794,7 +9062,9 @@
       <c r="H233" s="1">
         <v>20000</v>
       </c>
-      <c r="I233" s="1"/>
+      <c r="I233" s="1" t="s">
+        <v>663</v>
+      </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A234" s="1" t="s">
@@ -8879,7 +9149,9 @@
       <c r="H236" s="1">
         <v>20000</v>
       </c>
-      <c r="I236" s="1"/>
+      <c r="I236" s="1" t="s">
+        <v>673</v>
+      </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A237" s="1" t="s">
@@ -8906,7 +9178,9 @@
       <c r="H237" s="1">
         <v>20000</v>
       </c>
-      <c r="I237" s="1"/>
+      <c r="I237" s="1" t="s">
+        <v>664</v>
+      </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A238" s="1" t="s">
@@ -8933,7 +9207,9 @@
       <c r="H238" s="1">
         <v>20000</v>
       </c>
-      <c r="I238" s="1"/>
+      <c r="I238" s="1" t="s">
+        <v>665</v>
+      </c>
     </row>
     <row r="239" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A239" s="1" t="s">
@@ -8960,7 +9236,9 @@
       <c r="H239" s="1">
         <v>20000</v>
       </c>
-      <c r="I239" s="1"/>
+      <c r="I239" s="1" t="s">
+        <v>666</v>
+      </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A240" s="1" t="s">
@@ -9014,7 +9292,9 @@
       <c r="H241" s="1">
         <v>20000</v>
       </c>
-      <c r="I241" s="1"/>
+      <c r="I241" s="1" t="s">
+        <v>667</v>
+      </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A242" s="1" t="s">
@@ -9041,7 +9321,9 @@
       <c r="H242" s="1">
         <v>20000</v>
       </c>
-      <c r="I242" s="1"/>
+      <c r="I242" s="1" t="s">
+        <v>668</v>
+      </c>
     </row>
     <row r="243" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A243" s="1" t="s">
@@ -9068,7 +9350,9 @@
       <c r="H243" s="1">
         <v>20000</v>
       </c>
-      <c r="I243" s="1"/>
+      <c r="I243" s="1" t="s">
+        <v>669</v>
+      </c>
     </row>
     <row r="244" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A244" s="1" t="s">
@@ -9081,7 +9365,7 @@
         <v>399</v>
       </c>
       <c r="D244" s="1" t="s">
-        <v>141</v>
+        <v>14</v>
       </c>
       <c r="E244" s="1" t="s">
         <v>400</v>
@@ -9095,7 +9379,9 @@
       <c r="H244" s="1">
         <v>20000</v>
       </c>
-      <c r="I244" s="1"/>
+      <c r="I244" s="1" t="s">
+        <v>670</v>
+      </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A245" s="1" t="s">
@@ -9108,7 +9394,7 @@
         <v>399</v>
       </c>
       <c r="D245" s="1" t="s">
-        <v>141</v>
+        <v>14</v>
       </c>
       <c r="E245" s="1" t="s">
         <v>400</v>
@@ -9122,7 +9408,9 @@
       <c r="H245" s="1">
         <v>20000</v>
       </c>
-      <c r="I245" s="1"/>
+      <c r="I245" s="1" t="s">
+        <v>671</v>
+      </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A246" s="1" t="s">

</xml_diff>

<commit_message>
Pembaruan sistem RESIK BUMDes - 19/10/2026 13:38:46,73
</commit_message>
<xml_diff>
--- a/Template_Import_Pelanggan_RESIK_BUMDes.xlsx
+++ b/Template_Import_Pelanggan_RESIK_BUMDes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CODEX\antigrafity\revik bumdes v4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1FDC18C-6A0B-4B68-81A9-D585BC82BC53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58A615B2-90BA-4A9D-96FC-5142EE567A5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2116" uniqueCount="674">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2125" uniqueCount="682">
   <si>
     <t>Nama Pelanggan</t>
   </si>
@@ -2042,6 +2042,30 @@
   </si>
   <si>
     <t>7°19'33.77"S 110°28'00.61"E</t>
+  </si>
+  <si>
+    <t>7°19'33.90"S 110°27'56.25"E</t>
+  </si>
+  <si>
+    <t>7°19'23.28"S 110°28'05.08"E</t>
+  </si>
+  <si>
+    <t>7°19'21.27"S 110°28'08.04"E</t>
+  </si>
+  <si>
+    <t>7°19'24.52"S 110°28'07.41"E</t>
+  </si>
+  <si>
+    <t>7°19'23.10"S 110°28'04.46"E</t>
+  </si>
+  <si>
+    <t>7°19'24.37"S 110°28'21.41"E</t>
+  </si>
+  <si>
+    <t>7°19'24.73"S 110°28'21.05"E</t>
+  </si>
+  <si>
+    <t>7°20'08.94"S 110°27'53.98"E</t>
   </si>
 </sst>
 </file>
@@ -2057,12 +2081,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -2077,9 +2107,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5858,7 +5889,9 @@
       <c r="H121" s="1">
         <v>20000</v>
       </c>
-      <c r="I121" s="1"/>
+      <c r="I121" s="1" t="s">
+        <v>681</v>
+      </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A122" s="1" t="s">
@@ -9500,7 +9533,7 @@
       </c>
     </row>
     <row r="249" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A249" s="1" t="s">
+      <c r="A249" s="2" t="s">
         <v>453</v>
       </c>
       <c r="B249" s="1" t="s">
@@ -9551,10 +9584,12 @@
       <c r="H250" s="1">
         <v>20000</v>
       </c>
-      <c r="I250" s="1"/>
+      <c r="I250" s="1" t="s">
+        <v>677</v>
+      </c>
     </row>
     <row r="251" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A251" s="1" t="s">
+      <c r="A251" s="2" t="s">
         <v>457</v>
       </c>
       <c r="B251" s="1" t="s">
@@ -9578,7 +9613,9 @@
       <c r="H251" s="1">
         <v>20000</v>
       </c>
-      <c r="I251" s="1"/>
+      <c r="I251" s="1" t="s">
+        <v>678</v>
+      </c>
     </row>
     <row r="252" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A252" s="1" t="s">
@@ -9605,7 +9642,9 @@
       <c r="H252" s="1">
         <v>20000</v>
       </c>
-      <c r="I252" s="1"/>
+      <c r="I252" s="1" t="s">
+        <v>678</v>
+      </c>
     </row>
     <row r="253" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A253" s="1" t="s">
@@ -9632,7 +9671,9 @@
       <c r="H253" s="1">
         <v>20000</v>
       </c>
-      <c r="I253" s="1"/>
+      <c r="I253" s="1" t="s">
+        <v>675</v>
+      </c>
     </row>
     <row r="254" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A254" s="1" t="s">
@@ -9659,7 +9700,9 @@
       <c r="H254" s="1">
         <v>20000</v>
       </c>
-      <c r="I254" s="1"/>
+      <c r="I254" s="1" t="s">
+        <v>676</v>
+      </c>
     </row>
     <row r="255" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A255" s="1" t="s">
@@ -9744,7 +9787,9 @@
       <c r="H257" s="1">
         <v>20000</v>
       </c>
-      <c r="I257" s="1"/>
+      <c r="I257" s="1" t="s">
+        <v>679</v>
+      </c>
     </row>
     <row r="258" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A258" s="1" t="s">
@@ -9771,7 +9816,9 @@
       <c r="H258" s="1">
         <v>20000</v>
       </c>
-      <c r="I258" s="1"/>
+      <c r="I258" s="1" t="s">
+        <v>680</v>
+      </c>
     </row>
     <row r="259" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A259" s="1" t="s">
@@ -10080,7 +10127,9 @@
       <c r="H269" s="1">
         <v>20000</v>
       </c>
-      <c r="I269" s="1"/>
+      <c r="I269" s="1" t="s">
+        <v>674</v>
+      </c>
     </row>
     <row r="270" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A270" s="1" t="s">

</xml_diff>

<commit_message>
Pembaruan sistem RESIK BUMDes - 28/10/2026 21:41:45,59
</commit_message>
<xml_diff>
--- a/Template_Import_Pelanggan_RESIK_BUMDes.xlsx
+++ b/Template_Import_Pelanggan_RESIK_BUMDes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CODEX\antigrafity\revik bumdes v4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1621264-B04B-47CF-BFF4-A0127E372772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60C75EB4-0B59-4FE2-AB49-CEBDDEB1DE5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2125" uniqueCount="682">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2122" uniqueCount="684">
   <si>
     <t>Nama Pelanggan</t>
   </si>
@@ -2066,6 +2066,12 @@
   </si>
   <si>
     <t>7°20'08.94"S 110°27'53.98"E</t>
+  </si>
+  <si>
+    <t>08156526837</t>
+  </si>
+  <si>
+    <t>082137011432</t>
   </si>
 </sst>
 </file>
@@ -2107,10 +2113,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2454,6 +2461,7 @@
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.69921875" customWidth="1"/>
+    <col min="2" max="2" width="12.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
@@ -2785,8 +2793,8 @@
       <c r="A12" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>32</v>
+      <c r="B12" s="1">
+        <v>85642610551</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>18</v>
@@ -3276,9 +3284,7 @@
       <c r="A29" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>32</v>
-      </c>
+      <c r="B29" s="1"/>
       <c r="C29" s="1" t="s">
         <v>18</v>
       </c>
@@ -3421,8 +3427,8 @@
       <c r="A34" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B34" s="1" t="s">
-        <v>32</v>
+      <c r="B34" s="1">
+        <v>82134366414</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>18</v>
@@ -3537,8 +3543,8 @@
       <c r="A38" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B38" s="1" t="s">
-        <v>32</v>
+      <c r="B38" s="3" t="s">
+        <v>682</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>18</v>
@@ -3912,8 +3918,8 @@
       <c r="A51" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="B51" s="1" t="s">
-        <v>32</v>
+      <c r="B51" s="3" t="s">
+        <v>683</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>18</v>
@@ -3942,7 +3948,7 @@
         <v>521</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>32</v>
+        <v>96</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>18</v>

</xml_diff>